<commit_message>
Preserve manager attendance template print footer
</commit_message>
<xml_diff>
--- a/templates/export_templates/manager_attendance.xlsx
+++ b/templates/export_templates/manager_attendance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lewis\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{46EC5D01-3921-477E-8082-72549FBF927B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{235C17C9-52F7-4D5B-AE58-EE2A549A3C90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,23 +17,39 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">管理人员查询!$A$1:$M$109</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">管理人员查询!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="146">
+  <si>
+    <t>2026年4月份考勤记录</t>
+  </si>
+  <si>
+    <t>部   门</t>
+  </si>
   <si>
     <t>姓名</t>
   </si>
   <si>
+    <t>出勤天数</t>
+  </si>
+  <si>
+    <t>事/病假</t>
+  </si>
+  <si>
     <t>工伤</t>
   </si>
   <si>
     <t>出差</t>
   </si>
   <si>
+    <t>婚假</t>
+  </si>
+  <si>
     <t>丧假</t>
   </si>
   <si>
@@ -43,6 +59,9 @@
     <t>汇总</t>
   </si>
   <si>
+    <t>福利天数</t>
+  </si>
+  <si>
     <t>加班变化</t>
   </si>
   <si>
@@ -172,12 +191,18 @@
     <t>刘奕英</t>
   </si>
   <si>
+    <t>叶永健</t>
+  </si>
+  <si>
     <t>张俊峰</t>
   </si>
   <si>
     <t>17元</t>
   </si>
   <si>
+    <t>吴晓庆</t>
+  </si>
+  <si>
     <t>9元</t>
   </si>
   <si>
@@ -211,12 +236,18 @@
     <t>陈春娇</t>
   </si>
   <si>
+    <t>吴利蓉</t>
+  </si>
+  <si>
     <t>6元</t>
   </si>
   <si>
     <t>范春丽</t>
   </si>
   <si>
+    <t>吴苏娟</t>
+  </si>
+  <si>
     <t>吴逢平</t>
   </si>
   <si>
@@ -244,9 +275,15 @@
     <t>周晓芳</t>
   </si>
   <si>
+    <t>吴丽丽</t>
+  </si>
+  <si>
     <t>夏群</t>
   </si>
   <si>
+    <t>吴堂华</t>
+  </si>
+  <si>
     <t>扣1天</t>
   </si>
   <si>
@@ -289,9 +326,15 @@
     <t>扣0.5天，4元</t>
   </si>
   <si>
+    <t>刘春霞</t>
+  </si>
+  <si>
     <t>胡存寿</t>
   </si>
   <si>
+    <t>吴创海</t>
+  </si>
+  <si>
     <t>陈祥宇</t>
   </si>
   <si>
@@ -364,9 +407,6 @@
     <t>吴丽珍</t>
   </si>
   <si>
-    <t>安全管理部</t>
-  </si>
-  <si>
     <t>胡强</t>
   </si>
   <si>
@@ -379,9 +419,6 @@
     <t>吴尚华</t>
   </si>
   <si>
-    <t>设备动力部</t>
-  </si>
-  <si>
     <t>范春民</t>
   </si>
   <si>
@@ -419,87 +456,21 @@
   </si>
   <si>
     <t>吴家军</t>
-  </si>
-  <si>
-    <t>财务部</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>计划部</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>吴晓庆</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>吴苏娟</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>吴堂华</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>吴创海</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>出勤天数</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>事/病假</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>叶永健</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>吴利蓉</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>吴丽丽</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>刘春霞</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>福利天数</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>行政部</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>婚假</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>部门</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>（1）以上公布情况如有疑问、差错的地方，请各位员工到信息中心核对以便纠正。
 （2）凡请假、调休的，请假条与调休条必须在OA上提交，否则按旷工论处。
 （3）凡上班时间进出必须刷卡（除制度上规定人员外），不管私事或公事，都必须填写假条提交OA备案。</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026年4月份考勤记录</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026年4月</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -564,6 +535,13 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -591,7 +569,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -603,6 +581,39 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -651,15 +662,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -667,7 +669,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -678,146 +680,40 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="57" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="常规_2009年2月考勤" xfId="1" xr:uid="{72DA54AB-1636-4C0F-A84B-49E9ED9F9D51}"/>
+    <cellStyle name="常规_2009年2月考勤" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <color indexed="17"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="10"/>
-          <bgColor indexed="42"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <color indexed="60"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="10"/>
-          <bgColor indexed="29"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <color indexed="17"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="10"/>
-          <bgColor indexed="42"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <color indexed="60"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="10"/>
-          <bgColor indexed="29"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <color indexed="17"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="10"/>
-          <bgColor indexed="42"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <color indexed="60"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="10"/>
-          <bgColor indexed="29"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <color indexed="17"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="10"/>
-          <bgColor indexed="42"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <color indexed="60"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="10"/>
-          <bgColor indexed="29"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1151,69 +1047,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
       <c r="M1" s="7"/>
     </row>
     <row r="2" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>147</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>138</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>139</v>
+        <v>4</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>146</v>
+        <v>7</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>144</v>
+        <v>11</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="4" t="s">
-        <v>8</v>
+      <c r="A3" s="8" t="s">
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2">
         <v>26</v>
@@ -1246,11 +1142,9 @@
       <c r="M3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A4" s="5" t="s">
-        <v>132</v>
-      </c>
+      <c r="A4" s="9"/>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2">
         <v>22.5</v>
@@ -1283,11 +1177,9 @@
       <c r="M4" s="3"/>
     </row>
     <row r="5" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="A5" s="9"/>
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C5" s="2">
         <v>23.5</v>
@@ -1320,11 +1212,9 @@
       <c r="M5" s="3"/>
     </row>
     <row r="6" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="A6" s="9"/>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C6" s="2">
         <v>21.5</v>
@@ -1357,11 +1247,9 @@
       <c r="M6" s="3"/>
     </row>
     <row r="7" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="A7" s="9"/>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C7" s="2">
         <v>22</v>
@@ -1394,11 +1282,9 @@
       <c r="M7" s="3"/>
     </row>
     <row r="8" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="A8" s="10"/>
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C8" s="2">
         <v>24.5</v>
@@ -1431,11 +1317,11 @@
       <c r="M8" s="3"/>
     </row>
     <row r="9" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="5" t="s">
-        <v>15</v>
+      <c r="A9" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C9" s="2">
         <v>23</v>
@@ -1468,11 +1354,9 @@
       <c r="M9" s="3"/>
     </row>
     <row r="10" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A10" s="9"/>
       <c r="B10" s="2" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C10" s="2">
         <v>22.5</v>
@@ -1496,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="K10" s="2">
         <v>0</v>
@@ -1507,11 +1391,9 @@
       <c r="M10" s="3"/>
     </row>
     <row r="11" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A11" s="9"/>
       <c r="B11" s="2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C11" s="2">
         <v>22.5</v>
@@ -1544,11 +1426,9 @@
       <c r="M11" s="3"/>
     </row>
     <row r="12" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A12" s="9"/>
       <c r="B12" s="2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C12" s="2">
         <v>24</v>
@@ -1581,11 +1461,9 @@
       <c r="M12" s="3"/>
     </row>
     <row r="13" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A13" s="9"/>
       <c r="B13" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C13" s="2">
         <v>23</v>
@@ -1618,11 +1496,9 @@
       <c r="M13" s="3"/>
     </row>
     <row r="14" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A14" s="9"/>
       <c r="B14" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C14" s="2">
         <v>21.5</v>
@@ -1646,7 +1522,7 @@
         <v>4</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="K14" s="2">
         <v>0</v>
@@ -1655,15 +1531,13 @@
         <v>-1.5</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A15" s="9"/>
       <c r="B15" s="2" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C15" s="2">
         <v>23</v>
@@ -1696,11 +1570,9 @@
       <c r="M15" s="3"/>
     </row>
     <row r="16" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A16" s="9"/>
       <c r="B16" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C16" s="2">
         <v>24</v>
@@ -1733,11 +1605,9 @@
       <c r="M16" s="3"/>
     </row>
     <row r="17" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A17" s="9"/>
       <c r="B17" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C17" s="2">
         <v>23</v>
@@ -1770,11 +1640,9 @@
       <c r="M17" s="3"/>
     </row>
     <row r="18" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="5" t="s">
-        <v>133</v>
-      </c>
+      <c r="A18" s="9"/>
       <c r="B18" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C18" s="2">
         <v>22</v>
@@ -1798,7 +1666,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="K18" s="2">
         <v>0</v>
@@ -1807,15 +1675,13 @@
         <v>-1</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A19" s="9"/>
       <c r="B19" s="2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C19" s="2">
         <v>23</v>
@@ -1848,11 +1714,9 @@
       <c r="M19" s="3"/>
     </row>
     <row r="20" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="5" t="s">
-        <v>133</v>
-      </c>
+      <c r="A20" s="9"/>
       <c r="B20" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C20" s="2">
         <v>23</v>
@@ -1885,11 +1749,9 @@
       <c r="M20" s="3"/>
     </row>
     <row r="21" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A21" s="9"/>
       <c r="B21" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C21" s="2">
         <v>22.5</v>
@@ -1922,11 +1784,9 @@
       <c r="M21" s="3"/>
     </row>
     <row r="22" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A22" s="9"/>
       <c r="B22" s="2" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C22" s="2">
         <v>23</v>
@@ -1959,11 +1819,9 @@
       <c r="M22" s="3"/>
     </row>
     <row r="23" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A23" s="9"/>
       <c r="B23" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C23" s="2">
         <v>22</v>
@@ -1996,11 +1854,9 @@
       <c r="M23" s="3"/>
     </row>
     <row r="24" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="A24" s="9"/>
       <c r="B24" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C24" s="2">
         <v>23</v>
@@ -2033,11 +1889,9 @@
       <c r="M24" s="3"/>
     </row>
     <row r="25" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A25" s="9"/>
       <c r="B25" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C25" s="2">
         <v>22.5</v>
@@ -2070,11 +1924,9 @@
       <c r="M25" s="3"/>
     </row>
     <row r="26" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A26" s="9"/>
       <c r="B26" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C26" s="2">
         <v>22</v>
@@ -2107,11 +1959,9 @@
       <c r="M26" s="3"/>
     </row>
     <row r="27" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A27" s="9"/>
       <c r="B27" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C27" s="2">
         <v>23</v>
@@ -2144,11 +1994,9 @@
       <c r="M27" s="3"/>
     </row>
     <row r="28" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A28" s="10"/>
       <c r="B28" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C28" s="2">
         <v>22.5</v>
@@ -2172,7 +2020,7 @@
         <v>1</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="K28" s="2">
         <v>0</v>
@@ -2181,15 +2029,15 @@
         <v>-0.5</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="5" t="s">
-        <v>41</v>
+      <c r="A29" s="8" t="s">
+        <v>47</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C29" s="2">
         <v>22</v>
@@ -2222,11 +2070,9 @@
       <c r="M29" s="3"/>
     </row>
     <row r="30" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A30" s="9"/>
       <c r="B30" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C30" s="2">
         <v>23</v>
@@ -2259,11 +2105,9 @@
       <c r="M30" s="3"/>
     </row>
     <row r="31" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A31" s="9"/>
       <c r="B31" s="2" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C31" s="2">
         <v>21.5</v>
@@ -2287,7 +2131,7 @@
         <v>0</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="K31" s="2">
         <v>0</v>
@@ -2298,11 +2142,9 @@
       <c r="M31" s="3"/>
     </row>
     <row r="32" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A32" s="9"/>
       <c r="B32" s="2" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C32" s="2">
         <v>23</v>
@@ -2335,11 +2177,9 @@
       <c r="M32" s="3"/>
     </row>
     <row r="33" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A33" s="9"/>
       <c r="B33" s="2" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C33" s="2">
         <v>23</v>
@@ -2372,11 +2212,9 @@
       <c r="M33" s="3"/>
     </row>
     <row r="34" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A34" s="9"/>
       <c r="B34" s="2" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C34" s="2">
         <v>23</v>
@@ -2409,11 +2247,9 @@
       <c r="M34" s="3"/>
     </row>
     <row r="35" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="6" t="s">
-        <v>41</v>
-      </c>
+      <c r="A35" s="9"/>
       <c r="B35" s="2" t="s">
-        <v>140</v>
+        <v>55</v>
       </c>
       <c r="C35" s="2">
         <v>23</v>
@@ -2446,11 +2282,9 @@
       <c r="M35" s="3"/>
     </row>
     <row r="36" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="A36" s="9"/>
       <c r="B36" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C36" s="2">
         <v>23</v>
@@ -2474,7 +2308,7 @@
         <v>17</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="K36" s="2">
         <v>0</v>
@@ -2483,15 +2317,13 @@
         <v>0</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A37" s="9"/>
       <c r="B37" s="2" t="s">
-        <v>134</v>
+        <v>58</v>
       </c>
       <c r="C37" s="2">
         <v>23</v>
@@ -2515,7 +2347,7 @@
         <v>9</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="K37" s="2">
         <v>0</v>
@@ -2524,15 +2356,13 @@
         <v>0</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A38" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A38" s="9"/>
       <c r="B38" s="2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C38" s="2">
         <v>20.5</v>
@@ -2556,7 +2386,7 @@
         <v>15</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="K38" s="2">
         <v>0</v>
@@ -2565,15 +2395,13 @@
         <v>-2.5</v>
       </c>
       <c r="M38" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A39" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A39" s="9"/>
       <c r="B39" s="2" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="C39" s="2">
         <v>23</v>
@@ -2597,7 +2425,7 @@
         <v>3</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="K39" s="2">
         <v>0</v>
@@ -2606,15 +2434,13 @@
         <v>0</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A40" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A40" s="10"/>
       <c r="B40" s="2" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C40" s="2">
         <v>23</v>
@@ -2647,11 +2473,11 @@
       <c r="M40" s="3"/>
     </row>
     <row r="41" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A41" s="5" t="s">
-        <v>57</v>
+      <c r="A41" s="8" t="s">
+        <v>65</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C41" s="2">
         <v>23</v>
@@ -2684,11 +2510,9 @@
       <c r="M41" s="3"/>
     </row>
     <row r="42" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A42" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A42" s="9"/>
       <c r="B42" s="2" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C42" s="2">
         <v>23</v>
@@ -2721,11 +2545,9 @@
       <c r="M42" s="3"/>
     </row>
     <row r="43" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A43" s="9"/>
       <c r="B43" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C43" s="2">
         <v>23</v>
@@ -2758,11 +2580,9 @@
       <c r="M43" s="3"/>
     </row>
     <row r="44" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A44" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A44" s="9"/>
       <c r="B44" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="C44" s="2">
         <v>23.5</v>
@@ -2795,11 +2615,9 @@
       <c r="M44" s="3"/>
     </row>
     <row r="45" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A45" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A45" s="9"/>
       <c r="B45" s="2" t="s">
-        <v>141</v>
+        <v>70</v>
       </c>
       <c r="C45" s="2">
         <v>23</v>
@@ -2823,7 +2641,7 @@
         <v>6</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="K45" s="2">
         <v>0</v>
@@ -2832,15 +2650,13 @@
         <v>0</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A46" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A46" s="9"/>
       <c r="B46" s="2" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="C46" s="2">
         <v>23</v>
@@ -2873,11 +2689,9 @@
       <c r="M46" s="3"/>
     </row>
     <row r="47" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A47" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A47" s="9"/>
       <c r="B47" s="2" t="s">
-        <v>135</v>
+        <v>73</v>
       </c>
       <c r="C47" s="2">
         <v>23</v>
@@ -2901,7 +2715,7 @@
         <v>2</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="K47" s="2">
         <v>0</v>
@@ -2910,15 +2724,13 @@
         <v>0</v>
       </c>
       <c r="M47" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="48" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A48" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A48" s="9"/>
       <c r="B48" s="2" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C48" s="2">
         <v>23</v>
@@ -2951,11 +2763,9 @@
       <c r="M48" s="3"/>
     </row>
     <row r="49" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A49" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A49" s="9"/>
       <c r="B49" s="2" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C49" s="2">
         <v>23</v>
@@ -2988,11 +2798,9 @@
       <c r="M49" s="3"/>
     </row>
     <row r="50" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A50" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A50" s="9"/>
       <c r="B50" s="2" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="C50" s="2">
         <v>23</v>
@@ -3025,11 +2833,9 @@
       <c r="M50" s="3"/>
     </row>
     <row r="51" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A51" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A51" s="9"/>
       <c r="B51" s="2" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="C51" s="2">
         <v>23</v>
@@ -3062,11 +2868,9 @@
       <c r="M51" s="3"/>
     </row>
     <row r="52" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A52" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A52" s="10"/>
       <c r="B52" s="2" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C52" s="2">
         <v>23</v>
@@ -3099,11 +2903,11 @@
       <c r="M52" s="3"/>
     </row>
     <row r="53" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A53" s="5" t="s">
-        <v>69</v>
+      <c r="A53" s="8" t="s">
+        <v>79</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C53" s="2">
         <v>24</v>
@@ -3127,7 +2931,7 @@
         <v>2</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="K53" s="2">
         <v>0</v>
@@ -3136,15 +2940,13 @@
         <v>1</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A54" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A54" s="9"/>
       <c r="B54" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C54" s="2">
         <v>23</v>
@@ -3168,7 +2970,7 @@
         <v>3</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="K54" s="2">
         <v>0</v>
@@ -3177,15 +2979,13 @@
         <v>0</v>
       </c>
       <c r="M54" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="55" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A55" s="6" t="s">
-        <v>69</v>
-      </c>
+      <c r="A55" s="9"/>
       <c r="B55" s="2" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C55" s="2">
         <v>22.5</v>
@@ -3218,11 +3018,9 @@
       <c r="M55" s="3"/>
     </row>
     <row r="56" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A56" s="4" t="s">
-        <v>69</v>
-      </c>
+      <c r="A56" s="9"/>
       <c r="B56" s="2" t="s">
-        <v>142</v>
+        <v>83</v>
       </c>
       <c r="C56" s="2">
         <v>23</v>
@@ -3246,7 +3044,7 @@
         <v>3</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="K56" s="2">
         <v>0</v>
@@ -3255,15 +3053,13 @@
         <v>0</v>
       </c>
       <c r="M56" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="57" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A57" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A57" s="9"/>
       <c r="B57" s="2" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="C57" s="2">
         <v>22.5</v>
@@ -3296,11 +3092,9 @@
       <c r="M57" s="3"/>
     </row>
     <row r="58" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A58" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A58" s="9"/>
       <c r="B58" s="2" t="s">
-        <v>136</v>
+        <v>85</v>
       </c>
       <c r="C58" s="2">
         <v>17</v>
@@ -3324,7 +3118,7 @@
         <v>0</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="K58" s="2">
         <v>0</v>
@@ -3335,11 +3129,9 @@
       <c r="M58" s="3"/>
     </row>
     <row r="59" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A59" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A59" s="9"/>
       <c r="B59" s="2" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C59" s="2">
         <v>22.5</v>
@@ -3372,11 +3164,9 @@
       <c r="M59" s="3"/>
     </row>
     <row r="60" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A60" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A60" s="9"/>
       <c r="B60" s="2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="C60" s="2">
         <v>23</v>
@@ -3409,11 +3199,9 @@
       <c r="M60" s="3"/>
     </row>
     <row r="61" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A61" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A61" s="9"/>
       <c r="B61" s="2" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="C61" s="2">
         <v>6</v>
@@ -3437,7 +3225,7 @@
         <v>0</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="K61" s="2">
         <v>0</v>
@@ -3448,11 +3236,9 @@
       <c r="M61" s="3"/>
     </row>
     <row r="62" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A62" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A62" s="9"/>
       <c r="B62" s="2" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="C62" s="2">
         <v>23</v>
@@ -3485,11 +3271,9 @@
       <c r="M62" s="3"/>
     </row>
     <row r="63" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A63" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A63" s="9"/>
       <c r="B63" s="2" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="C63" s="2">
         <v>23</v>
@@ -3522,11 +3306,9 @@
       <c r="M63" s="3"/>
     </row>
     <row r="64" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A64" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A64" s="9"/>
       <c r="B64" s="2" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C64" s="2">
         <v>22</v>
@@ -3559,11 +3341,9 @@
       <c r="M64" s="3"/>
     </row>
     <row r="65" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A65" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A65" s="9"/>
       <c r="B65" s="2" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="C65" s="2">
         <v>23</v>
@@ -3596,11 +3376,9 @@
       <c r="M65" s="3"/>
     </row>
     <row r="66" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A66" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A66" s="9"/>
       <c r="B66" s="2" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C66" s="2">
         <v>23</v>
@@ -3633,11 +3411,9 @@
       <c r="M66" s="3"/>
     </row>
     <row r="67" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A67" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A67" s="9"/>
       <c r="B67" s="2" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="C67" s="2">
         <v>23</v>
@@ -3670,11 +3446,9 @@
       <c r="M67" s="3"/>
     </row>
     <row r="68" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A68" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A68" s="9"/>
       <c r="B68" s="2" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="C68" s="2">
         <v>22</v>
@@ -3707,11 +3481,9 @@
       <c r="M68" s="3"/>
     </row>
     <row r="69" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A69" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A69" s="9"/>
       <c r="B69" s="2" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="C69" s="2">
         <v>22.5</v>
@@ -3735,7 +3507,7 @@
         <v>4</v>
       </c>
       <c r="J69" s="2" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="K69" s="2">
         <v>0</v>
@@ -3744,15 +3516,13 @@
         <v>0</v>
       </c>
       <c r="M69" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A70" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A70" s="9"/>
       <c r="B70" s="2" t="s">
-        <v>143</v>
+        <v>100</v>
       </c>
       <c r="C70" s="2">
         <v>23</v>
@@ -3785,11 +3555,9 @@
       <c r="M70" s="3"/>
     </row>
     <row r="71" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A71" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A71" s="9"/>
       <c r="B71" s="2" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="C71" s="2">
         <v>23</v>
@@ -3822,11 +3590,9 @@
       <c r="M71" s="3"/>
     </row>
     <row r="72" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A72" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A72" s="9"/>
       <c r="B72" s="2" t="s">
-        <v>137</v>
+        <v>102</v>
       </c>
       <c r="C72" s="2">
         <v>23</v>
@@ -3859,11 +3625,9 @@
       <c r="M72" s="3"/>
     </row>
     <row r="73" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A73" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A73" s="9"/>
       <c r="B73" s="2" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="C73" s="2">
         <v>23</v>
@@ -3896,11 +3660,9 @@
       <c r="M73" s="3"/>
     </row>
     <row r="74" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A74" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A74" s="9"/>
       <c r="B74" s="2" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="C74" s="2">
         <v>21</v>
@@ -3924,7 +3686,7 @@
         <v>0</v>
       </c>
       <c r="J74" s="2" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="K74" s="2">
         <v>0</v>
@@ -3935,11 +3697,9 @@
       <c r="M74" s="3"/>
     </row>
     <row r="75" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A75" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A75" s="9"/>
       <c r="B75" s="2" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="C75" s="2">
         <v>22</v>
@@ -3972,11 +3732,9 @@
       <c r="M75" s="3"/>
     </row>
     <row r="76" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A76" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A76" s="9"/>
       <c r="B76" s="2" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="C76" s="2">
         <v>22.5</v>
@@ -4009,11 +3767,9 @@
       <c r="M76" s="3"/>
     </row>
     <row r="77" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A77" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A77" s="9"/>
       <c r="B77" s="2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C77" s="2">
         <v>22</v>
@@ -4037,7 +3793,7 @@
         <v>3</v>
       </c>
       <c r="J77" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="K77" s="2">
         <v>0</v>
@@ -4046,15 +3802,13 @@
         <v>-1</v>
       </c>
       <c r="M77" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="78" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A78" s="6" t="s">
-        <v>69</v>
-      </c>
+      <c r="A78" s="9"/>
       <c r="B78" s="2" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C78" s="2">
         <v>21</v>
@@ -4078,7 +3832,7 @@
         <v>0</v>
       </c>
       <c r="J78" s="2" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="K78" s="2">
         <v>0</v>
@@ -4089,11 +3843,9 @@
       <c r="M78" s="3"/>
     </row>
     <row r="79" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A79" s="8" t="s">
-        <v>69</v>
-      </c>
+      <c r="A79" s="10"/>
       <c r="B79" s="2" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="C79" s="2">
         <v>22</v>
@@ -4117,7 +3869,7 @@
         <v>0</v>
       </c>
       <c r="J79" s="2" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="K79" s="2">
         <v>0</v>
@@ -4129,10 +3881,10 @@
     </row>
     <row r="80" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A80" s="8" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="C80" s="2">
         <v>21</v>
@@ -4156,7 +3908,7 @@
         <v>3</v>
       </c>
       <c r="J80" s="2" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="K80" s="2">
         <v>0</v>
@@ -4165,15 +3917,13 @@
         <v>0</v>
       </c>
       <c r="M80" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="81" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A81" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A81" s="9"/>
       <c r="B81" s="2" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="C81" s="2">
         <v>23</v>
@@ -4206,11 +3956,9 @@
       <c r="M81" s="3"/>
     </row>
     <row r="82" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A82" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A82" s="9"/>
       <c r="B82" s="2" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="C82" s="2">
         <v>23</v>
@@ -4243,11 +3991,9 @@
       <c r="M82" s="3"/>
     </row>
     <row r="83" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A83" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A83" s="9"/>
       <c r="B83" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="C83" s="2">
         <v>23</v>
@@ -4280,11 +4026,9 @@
       <c r="M83" s="3"/>
     </row>
     <row r="84" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A84" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A84" s="9"/>
       <c r="B84" s="2" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="C84" s="2">
         <v>23</v>
@@ -4308,7 +4052,7 @@
         <v>4</v>
       </c>
       <c r="J84" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="K84" s="2">
         <v>0</v>
@@ -4317,15 +4061,13 @@
         <v>0</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="85" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A85" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A85" s="9"/>
       <c r="B85" s="2" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C85" s="2">
         <v>23</v>
@@ -4358,11 +4100,9 @@
       <c r="M85" s="3"/>
     </row>
     <row r="86" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A86" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A86" s="9"/>
       <c r="B86" s="2" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="C86" s="2">
         <v>19</v>
@@ -4386,7 +4126,7 @@
         <v>8</v>
       </c>
       <c r="J86" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="K86" s="2">
         <v>0</v>
@@ -4395,15 +4135,13 @@
         <v>-1</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="87" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A87" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A87" s="9"/>
       <c r="B87" s="2" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="C87" s="2">
         <v>23</v>
@@ -4427,7 +4165,7 @@
         <v>22</v>
       </c>
       <c r="J87" s="2" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="K87" s="2">
         <v>0</v>
@@ -4436,15 +4174,13 @@
         <v>0</v>
       </c>
       <c r="M87" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="88" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A88" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A88" s="9"/>
       <c r="B88" s="2" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C88" s="2">
         <v>23</v>
@@ -4468,7 +4204,7 @@
         <v>1</v>
       </c>
       <c r="J88" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="K88" s="2">
         <v>0</v>
@@ -4477,15 +4213,13 @@
         <v>0</v>
       </c>
       <c r="M88" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="89" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A89" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A89" s="9"/>
       <c r="B89" s="2" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C89" s="2">
         <v>25</v>
@@ -4509,7 +4243,7 @@
         <v>1</v>
       </c>
       <c r="J89" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="K89" s="2">
         <v>0</v>
@@ -4518,15 +4252,13 @@
         <v>2</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="90" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A90" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A90" s="9"/>
       <c r="B90" s="2" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C90" s="2">
         <v>24</v>
@@ -4559,11 +4291,9 @@
       <c r="M90" s="3"/>
     </row>
     <row r="91" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A91" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A91" s="9"/>
       <c r="B91" s="2" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C91" s="2">
         <v>22.5</v>
@@ -4587,7 +4317,7 @@
         <v>0</v>
       </c>
       <c r="J91" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="K91" s="2">
         <v>0</v>
@@ -4598,11 +4328,9 @@
       <c r="M91" s="3"/>
     </row>
     <row r="92" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A92" s="8" t="s">
-        <v>113</v>
-      </c>
+      <c r="A92" s="9"/>
       <c r="B92" s="2" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C92" s="2">
         <v>20</v>
@@ -4626,7 +4354,7 @@
         <v>0</v>
       </c>
       <c r="J92" s="2" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="K92" s="2">
         <v>0</v>
@@ -4637,11 +4365,9 @@
       <c r="M92" s="3"/>
     </row>
     <row r="93" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A93" s="8" t="s">
-        <v>113</v>
-      </c>
+      <c r="A93" s="9"/>
       <c r="B93" s="2" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="C93" s="2">
         <v>22</v>
@@ -4665,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="J93" s="2" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="K93" s="2">
         <v>0</v>
@@ -4676,11 +4402,9 @@
       <c r="M93" s="3"/>
     </row>
     <row r="94" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A94" s="8" t="s">
-        <v>113</v>
-      </c>
+      <c r="A94" s="10"/>
       <c r="B94" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C94" s="2">
         <v>23</v>
@@ -4714,10 +4438,10 @@
     </row>
     <row r="95" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="8" t="s">
-        <v>118</v>
+        <v>47</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="C95" s="2">
         <v>23</v>
@@ -4750,11 +4474,9 @@
       <c r="M95" s="3"/>
     </row>
     <row r="96" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A96" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A96" s="9"/>
       <c r="B96" s="2" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="C96" s="2">
         <v>21</v>
@@ -4778,7 +4500,7 @@
         <v>3</v>
       </c>
       <c r="J96" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="K96" s="2">
         <v>0</v>
@@ -4787,15 +4509,13 @@
         <v>-2</v>
       </c>
       <c r="M96" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="97" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A97" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A97" s="9"/>
       <c r="B97" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="C97" s="2">
         <v>23</v>
@@ -4828,11 +4548,9 @@
       <c r="M97" s="3"/>
     </row>
     <row r="98" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A98" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A98" s="9"/>
       <c r="B98" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C98" s="2">
         <v>23</v>
@@ -4856,7 +4574,7 @@
         <v>19</v>
       </c>
       <c r="J98" s="2" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="K98" s="2">
         <v>0</v>
@@ -4865,15 +4583,13 @@
         <v>0</v>
       </c>
       <c r="M98" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="99" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A99" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A99" s="9"/>
       <c r="B99" s="2" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="C99" s="2">
         <v>20.5</v>
@@ -4897,7 +4613,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="2" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="K99" s="2">
         <v>0</v>
@@ -4908,11 +4624,9 @@
       <c r="M99" s="3"/>
     </row>
     <row r="100" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A100" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A100" s="9"/>
       <c r="B100" s="2" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="C100" s="2">
         <v>23</v>
@@ -4945,11 +4659,9 @@
       <c r="M100" s="3"/>
     </row>
     <row r="101" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A101" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A101" s="9"/>
       <c r="B101" s="2" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C101" s="2">
         <v>23</v>
@@ -4982,11 +4694,9 @@
       <c r="M101" s="3"/>
     </row>
     <row r="102" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A102" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A102" s="9"/>
       <c r="B102" s="2" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="C102" s="2">
         <v>23</v>
@@ -5019,11 +4729,9 @@
       <c r="M102" s="3"/>
     </row>
     <row r="103" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A103" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A103" s="9"/>
       <c r="B103" s="2" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="C103" s="2">
         <v>23</v>
@@ -5056,11 +4764,9 @@
       <c r="M103" s="3"/>
     </row>
     <row r="104" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A104" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A104" s="9"/>
       <c r="B104" s="2" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="C104" s="2">
         <v>23</v>
@@ -5093,11 +4799,9 @@
       <c r="M104" s="3"/>
     </row>
     <row r="105" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A105" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A105" s="10"/>
       <c r="B105" s="2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C105" s="2">
         <v>20.5</v>
@@ -5121,7 +4825,7 @@
         <v>0</v>
       </c>
       <c r="J105" s="2" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="K105" s="2">
         <v>0</v>
@@ -5132,61 +4836,66 @@
       <c r="M105" s="3"/>
     </row>
     <row r="106" spans="1:13" ht="60" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A106" s="9"/>
-      <c r="B106" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="C106" s="10"/>
-      <c r="D106" s="10"/>
-      <c r="E106" s="10"/>
-      <c r="F106" s="10"/>
-      <c r="G106" s="10"/>
-      <c r="H106" s="10"/>
-      <c r="I106" s="10"/>
-      <c r="J106" s="10"/>
-      <c r="K106" s="10"/>
-      <c r="L106" s="10"/>
-      <c r="M106" s="10"/>
+      <c r="A106" s="4"/>
+      <c r="B106" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C106" s="15"/>
+      <c r="D106" s="15"/>
+      <c r="E106" s="15"/>
+      <c r="F106" s="15"/>
+      <c r="G106" s="15"/>
+      <c r="H106" s="15"/>
+      <c r="I106" s="15"/>
+      <c r="J106" s="15"/>
+      <c r="K106" s="15"/>
+      <c r="L106" s="15"/>
+      <c r="M106" s="15"/>
     </row>
     <row r="108" spans="1:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="J108" s="12" t="s">
-        <v>145</v>
+      <c r="J108" s="11" t="s">
+        <v>111</v>
       </c>
       <c r="K108" s="12"/>
       <c r="L108" s="12"/>
     </row>
-    <row r="109" spans="1:13" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="J109" s="13">
-        <v>46113</v>
-      </c>
-      <c r="K109" s="13"/>
-      <c r="L109" s="13"/>
+    <row r="109" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J109" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="K109" s="12"/>
+      <c r="L109" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="J109:L109"/>
+    <mergeCell ref="A80:A94"/>
+    <mergeCell ref="A41:A52"/>
     <mergeCell ref="B106:M106"/>
+    <mergeCell ref="A95:A105"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="A53:A79"/>
+    <mergeCell ref="A29:A40"/>
     <mergeCell ref="J108:L108"/>
-    <mergeCell ref="J109:L109"/>
-    <mergeCell ref="A79:A105"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A3:A17"/>
-    <mergeCell ref="A18:A23"/>
-    <mergeCell ref="A24:A35"/>
-    <mergeCell ref="A36:A55"/>
-    <mergeCell ref="A56:A78"/>
+    <mergeCell ref="A9:A28"/>
   </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <conditionalFormatting sqref="D3:D105">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J105">
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>第 &amp;P 页，共 &amp;N 页</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>